<commit_message>
MovitrentoLavis: Custom excelExport modificato su richiesta cliente
</commit_message>
<xml_diff>
--- a/PowerWeb/ExcelModels/ExportMovitrento.xlsx
+++ b/PowerWeb/ExcelModels/ExportMovitrento.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Winit.PowerWeb_old\PowerWeb\ExcelModels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EDFF70E-EE9E-4176-8856-71B2EC00F104}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB50D7B6-E98F-43EC-A1F6-40351333E57F}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2385" yWindow="495" windowWidth="22065" windowHeight="12750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Generale" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Generale!$B$1:$G$949</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Generale!$A$1:$G$10000</definedName>
   </definedNames>
   <calcPr calcId="152511"/>
 </workbook>
@@ -53424,6 +53424,7 @@
       <c r="D10000" s="1"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G10000" xr:uid="{2319889A-49DB-49CD-8422-880477008841}"/>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>